<commit_message>
fix-1 TSR sub prep update-1
</commit_message>
<xml_diff>
--- a/list.xlsx
+++ b/list.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\win10\Dropbox\Claude Projects\Visual Studio\Telecom Department\LMP Invoicing System\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\My Drive\Claude Projects\Visual Studio\Telecom Department\LMP Invoicing System\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6873BF91-F447-4974-801A-66F8541839BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{331865D8-81A1-428C-879F-4611C72F6EB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{A36F9A1A-2C4F-4B73-98F2-C72F17AB3B9E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A36F9A1A-2C4F-4B73-98F2-C72F17AB3B9E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Contractor</t>
   </si>
@@ -46,6 +46,9 @@
   </si>
   <si>
     <t>New Plan</t>
+  </si>
+  <si>
+    <t>Ikhtyar</t>
   </si>
 </sst>
 </file>
@@ -397,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{052A7D8C-112C-4888-B0C0-8E3D58144052}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
@@ -431,6 +434,11 @@
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>